<commit_message>
feat: add Chuseok, Mid-Autumn Festival and Tsukimi celebration banner and news
</commit_message>
<xml_diff>
--- a/kutlama takvimi.xlsx
+++ b/kutlama takvimi.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\2026 dünya\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30C0144D-C53F-4F73-A86A-F1D9AC5E0909}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2534A678-6BC2-4EC3-BDF1-48E9B36C04CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{00522D16-7C25-4C32-84FD-886C1952F0BD}"/>
   </bookViews>
@@ -617,12 +617,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -637,9 +643,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -978,6 +985,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="28" width="6.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:28" x14ac:dyDescent="0.25">
@@ -1064,7 +1072,7 @@
       </c>
     </row>
     <row r="2" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A2" s="1">
+      <c r="A2" s="2">
         <v>46272</v>
       </c>
       <c r="B2" t="s">

</xml_diff>